<commit_message>
Repair invalid worksheet XML element order in P001-P010 Excel and ZIP
</commit_message>
<xml_diff>
--- a/visualization/JXwork_P001-P010_Engineering_QA.xlsx
+++ b/visualization/JXwork_P001-P010_Engineering_QA.xlsx
@@ -360,11 +360,11 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:D16"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <autoFilter ref="A3:D16"/>
   <pageMargins left="0.35" right="0.35" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -707,6 +707,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:D16"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -717,7 +718,6 @@
     <hyperlink ref="D11" r:id="rId3" tooltip="打开同目录 resources 文件夹中的离线说明" display="查看补充资料"/>
     <hyperlink ref="D16" r:id="rId4" tooltip="打开同目录 resources 文件夹中的离线说明" display="查看补充资料"/>
   </hyperlinks>
-  <autoFilter ref="A3:D16"/>
   <pageMargins left="0.35" right="0.35" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -1060,6 +1060,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:D16"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -1067,7 +1068,6 @@
   <hyperlinks>
     <hyperlink ref="D4" r:id="rId1" tooltip="打开同目录 resources 文件夹中的离线说明" display="查看补充资料"/>
   </hyperlinks>
-  <autoFilter ref="A3:D16"/>
   <pageMargins left="0.35" right="0.35" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -1322,6 +1322,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:D12"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -1329,7 +1330,6 @@
   <hyperlinks>
     <hyperlink ref="D12" r:id="rId1" tooltip="打开同目录 resources 文件夹中的离线说明" display="查看补充资料"/>
   </hyperlinks>
-  <autoFilter ref="A3:D12"/>
   <pageMargins left="0.35" right="0.35" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -1672,11 +1672,11 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:D16"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
-  <autoFilter ref="A3:D16"/>
   <pageMargins left="0.35" right="0.35" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -1997,6 +1997,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:D15"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -2004,7 +2005,6 @@
   <hyperlinks>
     <hyperlink ref="D8" r:id="rId1" tooltip="打开同目录 resources 文件夹中的离线说明" display="查看补充资料"/>
   </hyperlinks>
-  <autoFilter ref="A3:D15"/>
   <pageMargins left="0.35" right="0.35" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -2325,6 +2325,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:D15"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -2333,7 +2334,6 @@
     <hyperlink ref="D6" r:id="rId1" tooltip="打开同目录 resources 文件夹中的离线说明" display="查看补充资料"/>
     <hyperlink ref="D15" r:id="rId2" tooltip="打开同目录 resources 文件夹中的离线说明" display="查看补充资料"/>
   </hyperlinks>
-  <autoFilter ref="A3:D15"/>
   <pageMargins left="0.35" right="0.35" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -2742,6 +2742,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:D19"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -2749,7 +2750,6 @@
   <hyperlinks>
     <hyperlink ref="D19" r:id="rId1" tooltip="打开同目录 resources 文件夹中的离线说明" display="查看补充资料"/>
   </hyperlinks>
-  <autoFilter ref="A3:D19"/>
   <pageMargins left="0.35" right="0.35" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -3180,6 +3180,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:D20"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -3187,7 +3188,6 @@
   <hyperlinks>
     <hyperlink ref="D20" r:id="rId1" tooltip="打开同目录 resources 文件夹中的离线说明" display="查看补充资料"/>
   </hyperlinks>
-  <autoFilter ref="A3:D20"/>
   <pageMargins left="0.35" right="0.35" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -3640,6 +3640,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:D21"/>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
@@ -3647,7 +3648,6 @@
   <hyperlinks>
     <hyperlink ref="D21" r:id="rId1" tooltip="打开同目录 resources 文件夹中的离线说明" display="查看补充资料"/>
   </hyperlinks>
-  <autoFilter ref="A3:D21"/>
   <pageMargins left="0.35" right="0.35" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>

</xml_diff>